<commit_message>
Add trend line charts to dashboard (issues, condition changes, all activity)
</commit_message>
<xml_diff>
--- a/data/equipment.xlsx
+++ b/data/equipment.xlsx
@@ -693,6 +693,9 @@
     <t>ROW-69</t>
   </si>
   <si>
+    <t>current-user</t>
+  </si>
+  <si>
     <t>58dd3900-a434-4f8a-892c-b6132c67e9c7</t>
   </si>
   <si>
@@ -1783,9 +1786,6 @@
   </si>
   <si>
     <t>1</t>
-  </si>
-  <si>
-    <t>current-user</t>
   </si>
   <si>
     <t>93422e06-4964-4837-900b-dd417f1751fe</t>
@@ -5840,19 +5840,19 @@
         <v>25</v>
       </c>
       <c r="M69" t="s">
-        <v>26</v>
+        <v>226</v>
       </c>
       <c r="N69" t="s">
         <v>25</v>
       </c>
       <c r="O69" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="P69">
-        <v>80.41514465745504</v>
+        <v>83.4375</v>
       </c>
       <c r="Q69">
-        <v>55.470527058186114</v>
+        <v>20.860047227249183</v>
       </c>
     </row>
     <row r="70" spans="1:17" x14ac:dyDescent="0.25">
@@ -5860,7 +5860,7 @@
         <v>59</v>
       </c>
       <c r="B70" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C70" t="s">
         <v>61</v>
@@ -5872,7 +5872,7 @@
         <v>21</v>
       </c>
       <c r="F70" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="G70">
         <v>1</v>
@@ -5893,19 +5893,19 @@
         <v>25</v>
       </c>
       <c r="M70" t="s">
-        <v>26</v>
+        <v>226</v>
       </c>
       <c r="N70" t="s">
         <v>25</v>
       </c>
       <c r="O70" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="P70">
-        <v>80.10248181222316</v>
+        <v>81.40625</v>
       </c>
       <c r="Q70">
-        <v>53.069746848577594</v>
+        <v>19.73531432042284</v>
       </c>
     </row>
     <row r="71" spans="1:17" x14ac:dyDescent="0.25">
@@ -5913,7 +5913,7 @@
         <v>59</v>
       </c>
       <c r="B71" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C71" t="s">
         <v>61</v>
@@ -5925,7 +5925,7 @@
         <v>21</v>
       </c>
       <c r="F71" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="G71">
         <v>1</v>
@@ -5946,19 +5946,19 @@
         <v>25</v>
       </c>
       <c r="M71" t="s">
-        <v>26</v>
+        <v>226</v>
       </c>
       <c r="N71" t="s">
         <v>25</v>
       </c>
       <c r="O71" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="P71">
-        <v>80.72780750268694</v>
+        <v>78.59375</v>
       </c>
       <c r="Q71">
-        <v>50.66896663896907</v>
+        <v>20.185207483153377</v>
       </c>
     </row>
     <row r="72" spans="1:17" x14ac:dyDescent="0.25">
@@ -5966,7 +5966,7 @@
         <v>59</v>
       </c>
       <c r="B72" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C72" t="s">
         <v>19</v>
@@ -5978,7 +5978,7 @@
         <v>21</v>
       </c>
       <c r="F72" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="G72">
         <v>0</v>
@@ -6005,7 +6005,7 @@
         <v>25</v>
       </c>
       <c r="O72" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="P72">
         <v>79.06027232811685</v>
@@ -6019,7 +6019,7 @@
         <v>59</v>
       </c>
       <c r="B73" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C73" t="s">
         <v>19</v>
@@ -6031,7 +6031,7 @@
         <v>21</v>
       </c>
       <c r="F73" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="G73">
         <v>1</v>
@@ -6058,7 +6058,7 @@
         <v>25</v>
       </c>
       <c r="O73" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="P73">
         <v>71.796875</v>
@@ -6069,10 +6069,10 @@
     </row>
     <row r="74" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B74" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C74" t="s">
         <v>19</v>
@@ -6084,7 +6084,7 @@
         <v>21</v>
       </c>
       <c r="F74" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="G74">
         <v>1</v>
@@ -6111,7 +6111,7 @@
         <v>25</v>
       </c>
       <c r="O74" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="P74">
         <v>9.128015944583767</v>
@@ -6122,10 +6122,10 @@
     </row>
     <row r="75" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B75" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C75" t="s">
         <v>19</v>
@@ -6137,7 +6137,7 @@
         <v>33</v>
       </c>
       <c r="F75" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="G75">
         <v>1</v>
@@ -6164,7 +6164,7 @@
         <v>25</v>
       </c>
       <c r="O75" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="P75">
         <v>10.066004480279442</v>
@@ -6175,10 +6175,10 @@
     </row>
     <row r="76" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B76" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C76" t="s">
         <v>19</v>
@@ -6190,7 +6190,7 @@
         <v>21</v>
       </c>
       <c r="F76" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="G76">
         <v>1</v>
@@ -6217,7 +6217,7 @@
         <v>25</v>
       </c>
       <c r="O76" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="P76">
         <v>11.6293187064389</v>
@@ -6228,10 +6228,10 @@
     </row>
     <row r="77" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B77" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C77" t="s">
         <v>19</v>
@@ -6243,7 +6243,7 @@
         <v>33</v>
       </c>
       <c r="F77" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="G77">
         <v>1</v>
@@ -6270,7 +6270,7 @@
         <v>25</v>
       </c>
       <c r="O77" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="P77">
         <v>12.254644396902684</v>
@@ -6281,10 +6281,10 @@
     </row>
     <row r="78" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B78" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C78" t="s">
         <v>19</v>
@@ -6296,7 +6296,7 @@
         <v>21</v>
       </c>
       <c r="F78" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="G78">
         <v>1</v>
@@ -6323,7 +6323,7 @@
         <v>25</v>
       </c>
       <c r="O78" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="P78">
         <v>16.944587075381058</v>
@@ -6334,10 +6334,10 @@
     </row>
     <row r="79" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B79" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C79" t="s">
         <v>19</v>
@@ -6349,7 +6349,7 @@
         <v>33</v>
       </c>
       <c r="F79" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="G79">
         <v>1</v>
@@ -6376,7 +6376,7 @@
         <v>25</v>
       </c>
       <c r="O79" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="P79">
         <v>18.299459404719254</v>
@@ -6387,10 +6387,10 @@
     </row>
     <row r="80" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B80" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C80" t="s">
         <v>19</v>
@@ -6402,7 +6402,7 @@
         <v>21</v>
       </c>
       <c r="F80" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="G80">
         <v>1</v>
@@ -6429,7 +6429,7 @@
         <v>25</v>
       </c>
       <c r="O80" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="P80">
         <v>20.90498311498502</v>
@@ -6440,10 +6440,10 @@
     </row>
     <row r="81" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B81" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C81" t="s">
         <v>19</v>
@@ -6455,7 +6455,7 @@
         <v>33</v>
       </c>
       <c r="F81" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="G81">
         <v>1</v>
@@ -6482,7 +6482,7 @@
         <v>25</v>
       </c>
       <c r="O81" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="P81">
         <v>22.885181134786997</v>
@@ -6493,10 +6493,10 @@
     </row>
     <row r="82" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B82" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C82" t="s">
         <v>19</v>
@@ -6508,7 +6508,7 @@
         <v>21</v>
       </c>
       <c r="F82" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="G82">
         <v>0</v>
@@ -6535,7 +6535,7 @@
         <v>25</v>
       </c>
       <c r="O82" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="P82">
         <v>23.09362303160826</v>
@@ -6546,10 +6546,10 @@
     </row>
     <row r="83" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B83" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C83" t="s">
         <v>19</v>
@@ -6561,7 +6561,7 @@
         <v>21</v>
       </c>
       <c r="F83" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="G83">
         <v>2</v>
@@ -6588,7 +6588,7 @@
         <v>25</v>
       </c>
       <c r="O83" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="P83">
         <v>28.200449503729157</v>
@@ -6599,10 +6599,10 @@
     </row>
     <row r="84" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B84" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C84" t="s">
         <v>19</v>
@@ -6614,7 +6614,7 @@
         <v>33</v>
       </c>
       <c r="F84" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="G84">
         <v>0</v>
@@ -6641,7 +6641,7 @@
         <v>25</v>
       </c>
       <c r="O84" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="P84">
         <v>27.366681916444115</v>
@@ -6652,10 +6652,10 @@
     </row>
     <row r="85" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B85" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C85" t="s">
         <v>19</v>
@@ -6667,7 +6667,7 @@
         <v>33</v>
       </c>
       <c r="F85" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="G85">
         <v>1</v>
@@ -6694,7 +6694,7 @@
         <v>25</v>
       </c>
       <c r="O85" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="P85">
         <v>29.13843803942483</v>
@@ -6705,10 +6705,10 @@
     </row>
     <row r="86" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B86" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C86" t="s">
         <v>19</v>
@@ -6720,7 +6720,7 @@
         <v>33</v>
       </c>
       <c r="F86" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="G86">
         <v>0</v>
@@ -6747,7 +6747,7 @@
         <v>25</v>
       </c>
       <c r="O86" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="P86">
         <v>32.05662459492248</v>
@@ -6758,10 +6758,10 @@
     </row>
     <row r="87" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B87" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C87" t="s">
         <v>19</v>
@@ -6773,7 +6773,7 @@
         <v>21</v>
       </c>
       <c r="F87" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="G87">
         <v>2</v>
@@ -6800,7 +6800,7 @@
         <v>25</v>
       </c>
       <c r="O87" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="P87">
         <v>33.41149692426068</v>
@@ -6811,10 +6811,10 @@
     </row>
     <row r="88" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B88" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C88" t="s">
         <v>19</v>
@@ -6826,7 +6826,7 @@
         <v>33</v>
       </c>
       <c r="F88" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="G88">
         <v>0</v>
@@ -6853,7 +6853,7 @@
         <v>25</v>
       </c>
       <c r="O88" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="P88">
         <v>35.28747399565203</v>
@@ -6864,10 +6864,10 @@
     </row>
     <row r="89" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B89" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C89" t="s">
         <v>19</v>
@@ -6879,7 +6879,7 @@
         <v>21</v>
       </c>
       <c r="F89" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="G89">
         <v>1</v>
@@ -6906,7 +6906,7 @@
         <v>25</v>
       </c>
       <c r="O89" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="P89">
         <v>6.5625</v>
@@ -6917,10 +6917,10 @@
     </row>
     <row r="90" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B90" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C90" t="s">
         <v>19</v>
@@ -6932,7 +6932,7 @@
         <v>21</v>
       </c>
       <c r="F90" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="G90">
         <v>1</v>
@@ -6959,7 +6959,7 @@
         <v>25</v>
       </c>
       <c r="O90" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="P90">
         <v>8.229166666666666</v>
@@ -6970,10 +6970,10 @@
     </row>
     <row r="91" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B91" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C91" t="s">
         <v>19</v>
@@ -6985,7 +6985,7 @@
         <v>21</v>
       </c>
       <c r="F91" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="G91">
         <v>1</v>
@@ -7012,7 +7012,7 @@
         <v>25</v>
       </c>
       <c r="O91" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="P91">
         <v>44.6875</v>
@@ -7023,10 +7023,10 @@
     </row>
     <row r="92" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B92" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C92" t="s">
         <v>19</v>
@@ -7038,7 +7038,7 @@
         <v>21</v>
       </c>
       <c r="F92" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="G92">
         <v>0</v>
@@ -7065,7 +7065,7 @@
         <v>25</v>
       </c>
       <c r="O92" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="P92">
         <v>42.604166666666664</v>
@@ -7076,10 +7076,10 @@
     </row>
     <row r="93" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B93" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C93" t="s">
         <v>19</v>
@@ -7091,7 +7091,7 @@
         <v>33</v>
       </c>
       <c r="F93" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="G93">
         <v>1</v>
@@ -7118,7 +7118,7 @@
         <v>25</v>
       </c>
       <c r="O93" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="P93">
         <v>37.916666666666664</v>
@@ -7129,10 +7129,10 @@
     </row>
     <row r="94" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B94" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C94" t="s">
         <v>19</v>
@@ -7144,7 +7144,7 @@
         <v>21</v>
       </c>
       <c r="F94" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="G94">
         <v>3</v>
@@ -7171,7 +7171,7 @@
         <v>25</v>
       </c>
       <c r="O94" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="P94">
         <v>36.354166666666664</v>
@@ -7182,10 +7182,10 @@
     </row>
     <row r="95" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B95" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C95" t="s">
         <v>19</v>
@@ -7197,7 +7197,7 @@
         <v>33</v>
       </c>
       <c r="F95" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="G95">
         <v>1</v>
@@ -7224,7 +7224,7 @@
         <v>25</v>
       </c>
       <c r="O95" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="P95">
         <v>35.208333333333336</v>
@@ -7235,10 +7235,10 @@
     </row>
     <row r="96" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B96" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C96" t="s">
         <v>19</v>
@@ -7250,7 +7250,7 @@
         <v>21</v>
       </c>
       <c r="F96" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="G96">
         <v>2</v>
@@ -7277,7 +7277,7 @@
         <v>25</v>
       </c>
       <c r="O96" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="P96">
         <v>32.395833333333336</v>
@@ -7288,10 +7288,10 @@
     </row>
     <row r="97" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B97" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C97" t="s">
         <v>19</v>
@@ -7303,7 +7303,7 @@
         <v>33</v>
       </c>
       <c r="F97" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="G97">
         <v>0</v>
@@ -7330,7 +7330,7 @@
         <v>25</v>
       </c>
       <c r="O97" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="P97">
         <v>32.1875</v>
@@ -7341,10 +7341,10 @@
     </row>
     <row r="98" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B98" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="C98" t="s">
         <v>19</v>
@@ -7356,7 +7356,7 @@
         <v>33</v>
       </c>
       <c r="F98" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="G98">
         <v>0</v>
@@ -7371,7 +7371,7 @@
         <v>131</v>
       </c>
       <c r="K98" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="L98" t="s">
         <v>25</v>
@@ -7383,7 +7383,7 @@
         <v>25</v>
       </c>
       <c r="O98" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="P98">
         <v>30.729166666666668</v>
@@ -7394,10 +7394,10 @@
     </row>
     <row r="99" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B99" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="C99" t="s">
         <v>19</v>
@@ -7409,7 +7409,7 @@
         <v>21</v>
       </c>
       <c r="F99" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="G99">
         <v>1</v>
@@ -7436,7 +7436,7 @@
         <v>25</v>
       </c>
       <c r="O99" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="P99">
         <v>28.229166666666668</v>
@@ -7447,10 +7447,10 @@
     </row>
     <row r="100" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B100" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C100" t="s">
         <v>19</v>
@@ -7462,7 +7462,7 @@
         <v>33</v>
       </c>
       <c r="F100" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="G100">
         <v>0</v>
@@ -7489,7 +7489,7 @@
         <v>25</v>
       </c>
       <c r="O100" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="P100">
         <v>28.645833333333332</v>
@@ -7500,10 +7500,10 @@
     </row>
     <row r="101" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B101" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C101" t="s">
         <v>19</v>
@@ -7515,7 +7515,7 @@
         <v>21</v>
       </c>
       <c r="F101" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G101">
         <v>2</v>
@@ -7542,7 +7542,7 @@
         <v>25</v>
       </c>
       <c r="O101" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="P101">
         <v>25.520833333333332</v>
@@ -7553,10 +7553,10 @@
     </row>
     <row r="102" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B102" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C102" t="s">
         <v>19</v>
@@ -7568,7 +7568,7 @@
         <v>33</v>
       </c>
       <c r="F102" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="G102">
         <v>0</v>
@@ -7595,7 +7595,7 @@
         <v>25</v>
       </c>
       <c r="O102" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="P102">
         <v>25.416666666666664</v>
@@ -7606,10 +7606,10 @@
     </row>
     <row r="103" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B103" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="C103" t="s">
         <v>19</v>
@@ -7621,7 +7621,7 @@
         <v>21</v>
       </c>
       <c r="F103" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="G103">
         <v>1</v>
@@ -7648,7 +7648,7 @@
         <v>25</v>
       </c>
       <c r="O103" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="P103">
         <v>23.020833333333332</v>
@@ -7659,10 +7659,10 @@
     </row>
     <row r="104" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B104" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="C104" t="s">
         <v>19</v>
@@ -7674,7 +7674,7 @@
         <v>21</v>
       </c>
       <c r="F104" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="G104">
         <v>2</v>
@@ -7701,7 +7701,7 @@
         <v>25</v>
       </c>
       <c r="O104" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="P104">
         <v>21.25</v>
@@ -7712,10 +7712,10 @@
     </row>
     <row r="105" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B105" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C105" t="s">
         <v>19</v>
@@ -7727,7 +7727,7 @@
         <v>21</v>
       </c>
       <c r="F105" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="G105">
         <v>1</v>
@@ -7754,7 +7754,7 @@
         <v>25</v>
       </c>
       <c r="O105" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="P105">
         <v>19.6875</v>
@@ -7765,10 +7765,10 @@
     </row>
     <row r="106" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B106" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C106" t="s">
         <v>19</v>
@@ -7780,7 +7780,7 @@
         <v>33</v>
       </c>
       <c r="F106" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G106">
         <v>1</v>
@@ -7807,7 +7807,7 @@
         <v>25</v>
       </c>
       <c r="O106" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="P106">
         <v>19.166666666666668</v>
@@ -7818,10 +7818,10 @@
     </row>
     <row r="107" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B107" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="C107" t="s">
         <v>19</v>
@@ -7833,7 +7833,7 @@
         <v>21</v>
       </c>
       <c r="F107" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="G107">
         <v>3</v>
@@ -7860,7 +7860,7 @@
         <v>25</v>
       </c>
       <c r="O107" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="P107">
         <v>16.145833333333336</v>
@@ -7871,10 +7871,10 @@
     </row>
     <row r="108" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B108" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="C108" t="s">
         <v>19</v>
@@ -7886,7 +7886,7 @@
         <v>33</v>
       </c>
       <c r="F108" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="G108">
         <v>1</v>
@@ -7913,7 +7913,7 @@
         <v>25</v>
       </c>
       <c r="O108" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="P108">
         <v>15</v>
@@ -7924,10 +7924,10 @@
     </row>
     <row r="109" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B109" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="C109" t="s">
         <v>19</v>
@@ -7939,7 +7939,7 @@
         <v>21</v>
       </c>
       <c r="F109" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="G109">
         <v>1</v>
@@ -7966,7 +7966,7 @@
         <v>25</v>
       </c>
       <c r="O109" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="P109">
         <v>13.750000000000002</v>
@@ -7977,10 +7977,10 @@
     </row>
     <row r="110" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B110" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C110" t="s">
         <v>19</v>
@@ -7992,7 +7992,7 @@
         <v>33</v>
       </c>
       <c r="F110" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="G110">
         <v>0</v>
@@ -8019,7 +8019,7 @@
         <v>25</v>
       </c>
       <c r="O110" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="P110">
         <v>13.229166666666666</v>
@@ -8030,10 +8030,10 @@
     </row>
     <row r="111" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B111" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C111" t="s">
         <v>19</v>
@@ -8045,7 +8045,7 @@
         <v>21</v>
       </c>
       <c r="F111" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="G111">
         <v>2</v>
@@ -8072,7 +8072,7 @@
         <v>25</v>
       </c>
       <c r="O111" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="P111">
         <v>9.625</v>
@@ -8083,10 +8083,10 @@
     </row>
     <row r="112" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B112" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C112" t="s">
         <v>19</v>
@@ -8098,7 +8098,7 @@
         <v>21</v>
       </c>
       <c r="F112" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="G112">
         <v>3</v>
@@ -8125,7 +8125,7 @@
         <v>25</v>
       </c>
       <c r="O112" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="P112">
         <v>15.5</v>
@@ -8136,10 +8136,10 @@
     </row>
     <row r="113" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B113" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="C113" t="s">
         <v>19</v>
@@ -8151,7 +8151,7 @@
         <v>21</v>
       </c>
       <c r="F113" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="G113">
         <v>1</v>
@@ -8178,7 +8178,7 @@
         <v>25</v>
       </c>
       <c r="O113" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="P113">
         <v>19.9375</v>
@@ -8189,10 +8189,10 @@
     </row>
     <row r="114" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="B114" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="C114" t="s">
         <v>19</v>
@@ -8204,7 +8204,7 @@
         <v>21</v>
       </c>
       <c r="F114" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="G114">
         <v>1</v>
@@ -8231,7 +8231,7 @@
         <v>25</v>
       </c>
       <c r="O114" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="P114">
         <v>42.5625</v>
@@ -8242,10 +8242,10 @@
     </row>
     <row r="115" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="B115" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="C115" t="s">
         <v>19</v>
@@ -8257,7 +8257,7 @@
         <v>21</v>
       </c>
       <c r="F115" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="G115">
         <v>0</v>
@@ -8284,7 +8284,7 @@
         <v>25</v>
       </c>
       <c r="O115" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="P115">
         <v>44.4375</v>
@@ -8295,10 +8295,10 @@
     </row>
     <row r="116" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="B116" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="C116" t="s">
         <v>19</v>
@@ -8310,7 +8310,7 @@
         <v>21</v>
       </c>
       <c r="F116" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="G116">
         <v>1</v>
@@ -8337,7 +8337,7 @@
         <v>25</v>
       </c>
       <c r="O116" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="P116">
         <v>41.875</v>
@@ -8348,10 +8348,10 @@
     </row>
     <row r="117" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="B117" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="C117" t="s">
         <v>19</v>
@@ -8363,7 +8363,7 @@
         <v>21</v>
       </c>
       <c r="F117" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="G117">
         <v>2</v>
@@ -8390,7 +8390,7 @@
         <v>25</v>
       </c>
       <c r="O117" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="P117">
         <v>39.625</v>
@@ -8401,10 +8401,10 @@
     </row>
     <row r="118" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="B118" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="C118" t="s">
         <v>19</v>
@@ -8416,7 +8416,7 @@
         <v>21</v>
       </c>
       <c r="F118" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="G118">
         <v>0</v>
@@ -8443,7 +8443,7 @@
         <v>25</v>
       </c>
       <c r="O118" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="P118">
         <v>37.5</v>
@@ -8454,10 +8454,10 @@
     </row>
     <row r="119" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="B119" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="C119" t="s">
         <v>19</v>
@@ -8469,7 +8469,7 @@
         <v>21</v>
       </c>
       <c r="F119" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="G119">
         <v>0</v>
@@ -8496,7 +8496,7 @@
         <v>25</v>
       </c>
       <c r="O119" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="P119">
         <v>37.5</v>
@@ -8507,10 +8507,10 @@
     </row>
     <row r="120" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="B120" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="C120" t="s">
         <v>19</v>
@@ -8522,7 +8522,7 @@
         <v>21</v>
       </c>
       <c r="F120" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="G120">
         <v>0</v>
@@ -8549,7 +8549,7 @@
         <v>25</v>
       </c>
       <c r="O120" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="P120">
         <v>35.25</v>
@@ -8560,10 +8560,10 @@
     </row>
     <row r="121" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="B121" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="C121" t="s">
         <v>19</v>
@@ -8575,7 +8575,7 @@
         <v>21</v>
       </c>
       <c r="F121" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="G121">
         <v>1</v>
@@ -8602,7 +8602,7 @@
         <v>25</v>
       </c>
       <c r="O121" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="P121">
         <v>35.25</v>
@@ -8613,10 +8613,10 @@
     </row>
     <row r="122" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="B122" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="C122" t="s">
         <v>19</v>
@@ -8628,7 +8628,7 @@
         <v>21</v>
       </c>
       <c r="F122" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="G122">
         <v>0</v>
@@ -8655,7 +8655,7 @@
         <v>25</v>
       </c>
       <c r="O122" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="P122">
         <v>27.8125</v>
@@ -8666,10 +8666,10 @@
     </row>
     <row r="123" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="B123" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C123" t="s">
         <v>19</v>
@@ -8681,7 +8681,7 @@
         <v>21</v>
       </c>
       <c r="F123" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="G123">
         <v>0</v>
@@ -8702,27 +8702,27 @@
         <v>25</v>
       </c>
       <c r="M123" t="s">
-        <v>26</v>
+        <v>226</v>
       </c>
       <c r="N123" t="s">
         <v>25</v>
       </c>
       <c r="O123" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="P123">
-        <v>28.812500000000004</v>
+        <v>66.875</v>
       </c>
       <c r="Q123">
-        <v>67.6114644714257</v>
+        <v>70.49825722691006</v>
       </c>
     </row>
     <row r="124" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="B124" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="C124" t="s">
         <v>19</v>
@@ -8734,7 +8734,7 @@
         <v>21</v>
       </c>
       <c r="F124" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="G124">
         <v>0</v>
@@ -8761,7 +8761,7 @@
         <v>25</v>
       </c>
       <c r="O124" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="P124">
         <v>21.1875</v>
@@ -8772,10 +8772,10 @@
     </row>
     <row r="125" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="B125" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="C125" t="s">
         <v>19</v>
@@ -8787,7 +8787,7 @@
         <v>33</v>
       </c>
       <c r="F125" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="G125">
         <v>1</v>
@@ -8814,7 +8814,7 @@
         <v>25</v>
       </c>
       <c r="O125" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="P125">
         <v>19.21875</v>
@@ -8825,10 +8825,10 @@
     </row>
     <row r="126" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="B126" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="C126" t="s">
         <v>19</v>
@@ -8840,7 +8840,7 @@
         <v>33</v>
       </c>
       <c r="F126" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="G126">
         <v>1</v>
@@ -8867,7 +8867,7 @@
         <v>25</v>
       </c>
       <c r="O126" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="P126">
         <v>19.21875</v>
@@ -8878,10 +8878,10 @@
     </row>
     <row r="127" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="B127" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="C127" t="s">
         <v>19</v>
@@ -8893,7 +8893,7 @@
         <v>33</v>
       </c>
       <c r="F127" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="G127">
         <v>0</v>
@@ -8920,7 +8920,7 @@
         <v>25</v>
       </c>
       <c r="O127" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="P127">
         <v>19.84375</v>
@@ -8931,10 +8931,10 @@
     </row>
     <row r="128" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="B128" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="C128" t="s">
         <v>19</v>
@@ -8946,7 +8946,7 @@
         <v>21</v>
       </c>
       <c r="F128" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="G128">
         <v>0</v>
@@ -8973,7 +8973,7 @@
         <v>25</v>
       </c>
       <c r="O128" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="P128">
         <v>19.21875</v>
@@ -8984,10 +8984,10 @@
     </row>
     <row r="129" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="B129" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="C129" t="s">
         <v>19</v>
@@ -8999,7 +8999,7 @@
         <v>33</v>
       </c>
       <c r="F129" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="G129">
         <v>0</v>
@@ -9026,7 +9026,7 @@
         <v>25</v>
       </c>
       <c r="O129" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="P129">
         <v>19.21875</v>
@@ -9037,10 +9037,10 @@
     </row>
     <row r="130" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="B130" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="C130" t="s">
         <v>19</v>
@@ -9052,7 +9052,7 @@
         <v>33</v>
       </c>
       <c r="F130" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="G130">
         <v>0</v>
@@ -9079,7 +9079,7 @@
         <v>25</v>
       </c>
       <c r="O130" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="P130">
         <v>19.21875</v>
@@ -9090,10 +9090,10 @@
     </row>
     <row r="131" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="B131" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="C131" t="s">
         <v>19</v>
@@ -9105,7 +9105,7 @@
         <v>33</v>
       </c>
       <c r="F131" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="G131">
         <v>1</v>
@@ -9132,7 +9132,7 @@
         <v>25</v>
       </c>
       <c r="O131" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="P131">
         <v>18.75</v>
@@ -9143,10 +9143,10 @@
     </row>
     <row r="132" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="B132" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="C132" t="s">
         <v>19</v>
@@ -9158,7 +9158,7 @@
         <v>21</v>
       </c>
       <c r="F132" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="G132">
         <v>2</v>
@@ -9185,7 +9185,7 @@
         <v>25</v>
       </c>
       <c r="O132" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="P132">
         <v>18.75</v>
@@ -9196,10 +9196,10 @@
     </row>
     <row r="133" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B133" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="C133" t="s">
         <v>19</v>
@@ -9211,7 +9211,7 @@
         <v>21</v>
       </c>
       <c r="F133" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="G133">
         <v>1</v>
@@ -9238,7 +9238,7 @@
         <v>25</v>
       </c>
       <c r="O133" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="P133">
         <v>49.461522979497786</v>
@@ -9249,10 +9249,10 @@
     </row>
     <row r="134" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B134" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="C134" t="s">
         <v>19</v>
@@ -9264,7 +9264,7 @@
         <v>21</v>
       </c>
       <c r="F134" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="G134">
         <v>0</v>
@@ -9291,7 +9291,7 @@
         <v>25</v>
       </c>
       <c r="O134" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="P134">
         <v>47.793987804927696</v>
@@ -9302,10 +9302,10 @@
     </row>
     <row r="135" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B135" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="C135" t="s">
         <v>19</v>
@@ -9317,7 +9317,7 @@
         <v>21</v>
       </c>
       <c r="F135" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="G135">
         <v>1</v>
@@ -9344,7 +9344,7 @@
         <v>25</v>
       </c>
       <c r="O135" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="P135">
         <v>54.35990755479742</v>
@@ -9355,10 +9355,10 @@
     </row>
     <row r="136" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B136" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C136" t="s">
         <v>19</v>
@@ -9370,7 +9370,7 @@
         <v>21</v>
       </c>
       <c r="F136" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="G136">
         <v>0</v>
@@ -9391,27 +9391,27 @@
         <v>25</v>
       </c>
       <c r="M136" t="s">
-        <v>26</v>
+        <v>226</v>
       </c>
       <c r="N136" t="s">
         <v>25</v>
       </c>
       <c r="O136" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="P136">
-        <v>45.60534788830445</v>
+        <v>54.84375</v>
       </c>
       <c r="Q136">
-        <v>15.857653599645467</v>
+        <v>24.684139110458737</v>
       </c>
     </row>
     <row r="137" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B137" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="C137" t="s">
         <v>19</v>
@@ -9423,7 +9423,7 @@
         <v>21</v>
       </c>
       <c r="F137" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="G137">
         <v>2</v>
@@ -9450,7 +9450,7 @@
         <v>25</v>
       </c>
       <c r="O137" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="P137">
         <v>57.395833333333336</v>
@@ -9461,10 +9461,10 @@
     </row>
     <row r="138" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B138" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="C138" t="s">
         <v>19</v>
@@ -9476,7 +9476,7 @@
         <v>21</v>
       </c>
       <c r="F138" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="G138">
         <v>1</v>
@@ -9503,7 +9503,7 @@
         <v>25</v>
       </c>
       <c r="O138" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="P138">
         <v>57.395833333333336</v>
@@ -9514,10 +9514,10 @@
     </row>
     <row r="139" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B139" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="C139" t="s">
         <v>19</v>
@@ -9529,7 +9529,7 @@
         <v>21</v>
       </c>
       <c r="F139" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="G139">
         <v>1</v>
@@ -9550,27 +9550,27 @@
         <v>25</v>
       </c>
       <c r="M139" t="s">
-        <v>26</v>
+        <v>226</v>
       </c>
       <c r="N139" t="s">
         <v>25</v>
       </c>
       <c r="O139" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="P139">
-        <v>42.79138228121743</v>
+        <v>61.09375</v>
       </c>
       <c r="Q139">
-        <v>17.65823875685186</v>
+        <v>23.78435278499767</v>
       </c>
     </row>
     <row r="140" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B140" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="C140" t="s">
         <v>19</v>
@@ -9582,7 +9582,7 @@
         <v>21</v>
       </c>
       <c r="F140" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="G140">
         <v>0</v>
@@ -9603,27 +9603,27 @@
         <v>25</v>
       </c>
       <c r="M140" t="s">
-        <v>26</v>
+        <v>226</v>
       </c>
       <c r="N140" t="s">
         <v>25</v>
       </c>
       <c r="O140" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="P140">
-        <v>43.93781271373437</v>
+        <v>69.84375</v>
       </c>
       <c r="Q140">
-        <v>15.107409784142803</v>
+        <v>25.358978854554543</v>
       </c>
     </row>
     <row r="141" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="B141" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="C141" t="s">
         <v>19</v>
@@ -9635,7 +9635,7 @@
         <v>33</v>
       </c>
       <c r="F141" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="G141">
         <v>1</v>
@@ -9650,7 +9650,7 @@
         <v>131</v>
       </c>
       <c r="K141" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="L141" t="s">
         <v>25</v>
@@ -9662,7 +9662,7 @@
         <v>25</v>
       </c>
       <c r="O141" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="P141">
         <v>60</v>
@@ -9673,10 +9673,10 @@
     </row>
     <row r="142" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="B142" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="C142" t="s">
         <v>19</v>
@@ -9688,7 +9688,7 @@
         <v>21</v>
       </c>
       <c r="F142" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="G142">
         <v>0</v>
@@ -9700,10 +9700,10 @@
         <v>24</v>
       </c>
       <c r="J142" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="K142" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="L142" t="s">
         <v>25</v>
@@ -9715,7 +9715,7 @@
         <v>25</v>
       </c>
       <c r="O142" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="P142">
         <v>60</v>
@@ -9726,10 +9726,10 @@
     </row>
     <row r="143" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="B143" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="C143" t="s">
         <v>19</v>
@@ -9741,7 +9741,7 @@
         <v>21</v>
       </c>
       <c r="F143" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="G143">
         <v>0</v>
@@ -9753,10 +9753,10 @@
         <v>24</v>
       </c>
       <c r="J143" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="K143" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="L143" t="s">
         <v>25</v>
@@ -9768,7 +9768,7 @@
         <v>25</v>
       </c>
       <c r="O143" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="P143">
         <v>60</v>
@@ -9779,10 +9779,10 @@
     </row>
     <row r="144" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="B144" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="C144" t="s">
         <v>19</v>
@@ -9794,7 +9794,7 @@
         <v>33</v>
       </c>
       <c r="F144" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="G144">
         <v>1</v>
@@ -9806,10 +9806,10 @@
         <v>30</v>
       </c>
       <c r="J144" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="K144" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="L144" t="s">
         <v>25</v>
@@ -9821,7 +9821,7 @@
         <v>25</v>
       </c>
       <c r="O144" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="P144">
         <v>58.828125</v>
@@ -9832,10 +9832,10 @@
     </row>
     <row r="145" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="B145" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="C145" t="s">
         <v>19</v>
@@ -9847,7 +9847,7 @@
         <v>33</v>
       </c>
       <c r="F145" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="G145">
         <v>1</v>
@@ -9859,7 +9859,7 @@
         <v>30</v>
       </c>
       <c r="J145" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="K145" t="s">
         <v>25</v>
@@ -9874,7 +9874,7 @@
         <v>25</v>
       </c>
       <c r="O145" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="P145">
         <v>56.32812499999999</v>
@@ -9885,7 +9885,7 @@
     </row>
     <row r="146" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="B146" t="s">
         <v>168</v>
@@ -9900,7 +9900,7 @@
         <v>33</v>
       </c>
       <c r="F146" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="G146">
         <v>1</v>
@@ -9912,7 +9912,7 @@
         <v>30</v>
       </c>
       <c r="J146" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="K146" t="s">
         <v>25</v>
@@ -9927,7 +9927,7 @@
         <v>25</v>
       </c>
       <c r="O146" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="P146">
         <v>53.515625</v>
@@ -9938,10 +9938,10 @@
     </row>
     <row r="147" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="B147" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="C147" t="s">
         <v>19</v>
@@ -9953,7 +9953,7 @@
         <v>21</v>
       </c>
       <c r="F147" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="G147">
         <v>0</v>
@@ -9965,7 +9965,7 @@
         <v>30</v>
       </c>
       <c r="J147" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="K147" t="s">
         <v>25</v>
@@ -9974,27 +9974,27 @@
         <v>25</v>
       </c>
       <c r="M147" t="s">
-        <v>26</v>
+        <v>226</v>
       </c>
       <c r="N147" t="s">
         <v>25</v>
       </c>
       <c r="O147" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="P147">
-        <v>44.45891745578752</v>
+        <v>49.895833333333336</v>
       </c>
       <c r="Q147">
-        <v>18.858628861656122</v>
+        <v>48.21915293593007</v>
       </c>
     </row>
     <row r="148" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="B148" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="C148" t="s">
         <v>19</v>
@@ -10006,7 +10006,7 @@
         <v>21</v>
       </c>
       <c r="F148" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="G148">
         <v>0</v>
@@ -10018,7 +10018,7 @@
         <v>24</v>
       </c>
       <c r="J148" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K148" t="s">
         <v>25</v>
@@ -10033,7 +10033,7 @@
         <v>25</v>
       </c>
       <c r="O148" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="P148">
         <v>27.421875</v>
@@ -10044,10 +10044,10 @@
     </row>
     <row r="149" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="B149" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="C149" t="s">
         <v>19</v>
@@ -10059,7 +10059,7 @@
         <v>33</v>
       </c>
       <c r="F149" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="G149">
         <v>0</v>
@@ -10071,7 +10071,7 @@
         <v>24</v>
       </c>
       <c r="J149" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="K149" t="s">
         <v>25</v>
@@ -10086,7 +10086,7 @@
         <v>25</v>
       </c>
       <c r="O149" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="P149">
         <v>27.421875</v>
@@ -10097,10 +10097,10 @@
     </row>
     <row r="150" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="B150" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="C150" t="s">
         <v>19</v>
@@ -10112,7 +10112,7 @@
         <v>21</v>
       </c>
       <c r="F150" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="G150">
         <v>0</v>
@@ -10124,7 +10124,7 @@
         <v>24</v>
       </c>
       <c r="J150" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="K150" t="s">
         <v>25</v>
@@ -10139,7 +10139,7 @@
         <v>25</v>
       </c>
       <c r="O150" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="P150">
         <v>27.421875</v>
@@ -10150,10 +10150,10 @@
     </row>
     <row r="151" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="B151" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="C151" t="s">
         <v>19</v>
@@ -10165,7 +10165,7 @@
         <v>33</v>
       </c>
       <c r="F151" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="G151">
         <v>0</v>
@@ -10177,7 +10177,7 @@
         <v>24</v>
       </c>
       <c r="J151" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="K151" t="s">
         <v>25</v>
@@ -10192,7 +10192,7 @@
         <v>25</v>
       </c>
       <c r="O151" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="P151">
         <v>27.421875</v>
@@ -10203,10 +10203,10 @@
     </row>
     <row r="152" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="B152" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="C152" t="s">
         <v>19</v>
@@ -10218,7 +10218,7 @@
         <v>21</v>
       </c>
       <c r="F152" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="G152">
         <v>1</v>
@@ -10230,7 +10230,7 @@
         <v>30</v>
       </c>
       <c r="J152" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="K152" t="s">
         <v>25</v>
@@ -10245,7 +10245,7 @@
         <v>25</v>
       </c>
       <c r="O152" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="P152">
         <v>56.32812499999999</v>
@@ -10256,10 +10256,10 @@
     </row>
     <row r="153" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="B153" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="C153" t="s">
         <v>61</v>
@@ -10271,7 +10271,7 @@
         <v>21</v>
       </c>
       <c r="F153" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="G153">
         <v>1</v>
@@ -10283,7 +10283,7 @@
         <v>144</v>
       </c>
       <c r="J153" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K153" t="s">
         <v>25</v>
@@ -10298,7 +10298,7 @@
         <v>25</v>
       </c>
       <c r="O153" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="P153">
         <v>9.753341635047551</v>
@@ -10309,7 +10309,7 @@
     </row>
     <row r="154" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="B154" t="s">
         <v>168</v>
@@ -10324,7 +10324,7 @@
         <v>21</v>
       </c>
       <c r="F154" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="G154">
         <v>1</v>
@@ -10336,7 +10336,7 @@
         <v>30</v>
       </c>
       <c r="J154" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K154" t="s">
         <v>25</v>
@@ -10351,7 +10351,7 @@
         <v>25</v>
       </c>
       <c r="O154" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="P154">
         <v>6.6267131827286345</v>
@@ -10362,10 +10362,10 @@
     </row>
     <row r="155" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="B155" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="C155" t="s">
         <v>61</v>
@@ -10377,7 +10377,7 @@
         <v>21</v>
       </c>
       <c r="F155" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="G155">
         <v>1</v>
@@ -10389,7 +10389,7 @@
         <v>30</v>
       </c>
       <c r="J155" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K155" t="s">
         <v>25</v>
@@ -10404,7 +10404,7 @@
         <v>25</v>
       </c>
       <c r="O155" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="P155">
         <v>7.043596976371156</v>
@@ -10415,10 +10415,10 @@
     </row>
     <row r="156" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="B156" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="C156" t="s">
         <v>61</v>
@@ -10430,7 +10430,7 @@
         <v>21</v>
       </c>
       <c r="F156" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="G156">
         <v>1</v>
@@ -10442,7 +10442,7 @@
         <v>30</v>
       </c>
       <c r="J156" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K156" t="s">
         <v>25</v>
@@ -10457,7 +10457,7 @@
         <v>25</v>
       </c>
       <c r="O156" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="P156">
         <v>6.835155079549896</v>
@@ -10468,10 +10468,10 @@
     </row>
     <row r="157" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="B157" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="C157" t="s">
         <v>61</v>
@@ -10483,7 +10483,7 @@
         <v>21</v>
       </c>
       <c r="F157" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="G157">
         <v>1</v>
@@ -10495,7 +10495,7 @@
         <v>30</v>
       </c>
       <c r="J157" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K157" t="s">
         <v>25</v>
@@ -10510,7 +10510,7 @@
         <v>25</v>
       </c>
       <c r="O157" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="P157">
         <v>10.482888273921965</v>
@@ -10521,10 +10521,10 @@
     </row>
     <row r="158" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="B158" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="C158" t="s">
         <v>61</v>
@@ -10536,7 +10536,7 @@
         <v>33</v>
       </c>
       <c r="F158" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="G158">
         <v>1</v>
@@ -10548,10 +10548,10 @@
         <v>30</v>
       </c>
       <c r="J158" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K158" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="L158" t="s">
         <v>25</v>
@@ -10563,7 +10563,7 @@
         <v>25</v>
       </c>
       <c r="O158" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="P158">
         <v>6.209829389086113</v>
@@ -10574,10 +10574,10 @@
     </row>
     <row r="159" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="B159" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="C159" t="s">
         <v>61</v>
@@ -10589,7 +10589,7 @@
         <v>21</v>
       </c>
       <c r="F159" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="G159">
         <v>1</v>
@@ -10601,7 +10601,7 @@
         <v>30</v>
       </c>
       <c r="J159" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K159" t="s">
         <v>25</v>
@@ -10616,7 +10616,7 @@
         <v>25</v>
       </c>
       <c r="O159" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="P159">
         <v>4.2296313692841325</v>
@@ -10627,10 +10627,10 @@
     </row>
     <row r="160" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="B160" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="C160" t="s">
         <v>61</v>
@@ -10642,7 +10642,7 @@
         <v>21</v>
       </c>
       <c r="F160" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="G160">
         <v>1</v>
@@ -10654,7 +10654,7 @@
         <v>30</v>
       </c>
       <c r="J160" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K160" t="s">
         <v>25</v>
@@ -10669,7 +10669,7 @@
         <v>25</v>
       </c>
       <c r="O160" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="P160">
         <v>10.170225428690074</v>
@@ -10680,10 +10680,10 @@
     </row>
     <row r="161" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="B161" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="C161" t="s">
         <v>61</v>
@@ -10695,7 +10695,7 @@
         <v>21</v>
       </c>
       <c r="F161" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="G161">
         <v>1</v>
@@ -10707,7 +10707,7 @@
         <v>30</v>
       </c>
       <c r="J161" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K161" t="s">
         <v>25</v>
@@ -10722,7 +10722,7 @@
         <v>25</v>
       </c>
       <c r="O161" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="P161">
         <v>10.066004480279442</v>
@@ -10733,10 +10733,10 @@
     </row>
     <row r="162" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="B162" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="C162" t="s">
         <v>61</v>
@@ -10748,7 +10748,7 @@
         <v>21</v>
       </c>
       <c r="F162" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="G162">
         <v>1</v>
@@ -10760,7 +10760,7 @@
         <v>30</v>
       </c>
       <c r="J162" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K162" t="s">
         <v>25</v>
@@ -10775,7 +10775,7 @@
         <v>25</v>
       </c>
       <c r="O162" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="P162">
         <v>7.66892266683494</v>
@@ -10786,10 +10786,10 @@
     </row>
     <row r="163" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="B163" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="C163" t="s">
         <v>61</v>
@@ -10801,7 +10801,7 @@
         <v>21</v>
       </c>
       <c r="F163" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="G163">
         <v>1</v>
@@ -10813,7 +10813,7 @@
         <v>30</v>
       </c>
       <c r="J163" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K163" t="s">
         <v>25</v>
@@ -10828,7 +10828,7 @@
         <v>25</v>
       </c>
       <c r="O163" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="P163">
         <v>9.0625</v>
@@ -10839,10 +10839,10 @@
     </row>
     <row r="164" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="B164" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="C164" t="s">
         <v>61</v>
@@ -10854,7 +10854,7 @@
         <v>21</v>
       </c>
       <c r="F164" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="G164">
         <v>1</v>
@@ -10866,7 +10866,7 @@
         <v>30</v>
       </c>
       <c r="J164" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K164" t="s">
         <v>25</v>
@@ -10881,7 +10881,7 @@
         <v>25</v>
       </c>
       <c r="O164" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="P164">
         <v>9.0625</v>
@@ -10892,10 +10892,10 @@
     </row>
     <row r="165" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="B165" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="C165" t="s">
         <v>61</v>
@@ -10907,7 +10907,7 @@
         <v>21</v>
       </c>
       <c r="F165" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="G165">
         <v>0</v>
@@ -10919,7 +10919,7 @@
         <v>24</v>
       </c>
       <c r="J165" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K165" t="s">
         <v>25</v>
@@ -10934,7 +10934,7 @@
         <v>25</v>
       </c>
       <c r="O165" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="P165">
         <v>7.147817924781788</v>
@@ -10945,10 +10945,10 @@
     </row>
     <row r="166" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="B166" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="C166" t="s">
         <v>61</v>
@@ -10960,7 +10960,7 @@
         <v>21</v>
       </c>
       <c r="F166" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="G166">
         <v>1</v>
@@ -10972,10 +10972,10 @@
         <v>24</v>
       </c>
       <c r="J166" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K166" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="L166" t="s">
         <v>25</v>
@@ -10987,7 +10987,7 @@
         <v>25</v>
       </c>
       <c r="O166" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="P166">
         <v>8.919574047762506</v>
@@ -11001,7 +11001,7 @@
         <v>59</v>
       </c>
       <c r="B167" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="C167" t="s">
         <v>19</v>
@@ -11013,7 +11013,7 @@
         <v>33</v>
       </c>
       <c r="F167" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="G167">
         <v>1</v>
@@ -11025,7 +11025,7 @@
         <v>30</v>
       </c>
       <c r="J167" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K167" t="s">
         <v>25</v>
@@ -11040,7 +11040,7 @@
         <v>25</v>
       </c>
       <c r="O167" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="P167">
         <v>82.65625</v>
@@ -11054,7 +11054,7 @@
         <v>59</v>
       </c>
       <c r="B168" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="C168" t="s">
         <v>19</v>
@@ -11066,7 +11066,7 @@
         <v>21</v>
       </c>
       <c r="F168" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="G168">
         <v>1</v>
@@ -11078,7 +11078,7 @@
         <v>30</v>
       </c>
       <c r="J168" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K168" t="s">
         <v>25</v>
@@ -11093,7 +11093,7 @@
         <v>25</v>
       </c>
       <c r="O168" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="P168">
         <v>83.125</v>
@@ -11107,7 +11107,7 @@
         <v>59</v>
       </c>
       <c r="B169" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="C169" t="s">
         <v>19</v>
@@ -11119,7 +11119,7 @@
         <v>21</v>
       </c>
       <c r="F169" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="G169">
         <v>0</v>
@@ -11131,7 +11131,7 @@
         <v>24</v>
       </c>
       <c r="J169" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K169" t="s">
         <v>25</v>
@@ -11140,19 +11140,19 @@
         <v>25</v>
       </c>
       <c r="M169" t="s">
-        <v>26</v>
+        <v>226</v>
       </c>
       <c r="N169" t="s">
         <v>25</v>
       </c>
       <c r="O169" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="P169">
-        <v>78.43494822793853</v>
+        <v>76.40625</v>
       </c>
       <c r="Q169">
-        <v>30.962563181619906</v>
+        <v>31.432536551416785</v>
       </c>
     </row>
     <row r="170" spans="1:17" x14ac:dyDescent="0.25">
@@ -11160,7 +11160,7 @@
         <v>59</v>
       </c>
       <c r="B170" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="C170" t="s">
         <v>19</v>
@@ -11172,7 +11172,7 @@
         <v>21</v>
       </c>
       <c r="F170" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="G170">
         <v>2</v>
@@ -11184,7 +11184,7 @@
         <v>30</v>
       </c>
       <c r="J170" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K170" t="s">
         <v>25</v>
@@ -11199,7 +11199,7 @@
         <v>25</v>
       </c>
       <c r="O170" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="P170">
         <v>81.40625</v>
@@ -11213,7 +11213,7 @@
         <v>59</v>
       </c>
       <c r="B171" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="C171" t="s">
         <v>19</v>
@@ -11225,7 +11225,7 @@
         <v>21</v>
       </c>
       <c r="F171" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="G171">
         <v>0</v>
@@ -11237,7 +11237,7 @@
         <v>24</v>
       </c>
       <c r="J171" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K171" t="s">
         <v>25</v>
@@ -11252,7 +11252,7 @@
         <v>25</v>
       </c>
       <c r="O171" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="P171">
         <v>82.734375</v>
@@ -11266,7 +11266,7 @@
         <v>59</v>
       </c>
       <c r="B172" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="C172" t="s">
         <v>19</v>
@@ -11278,7 +11278,7 @@
         <v>21</v>
       </c>
       <c r="F172" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="G172">
         <v>0</v>
@@ -11290,7 +11290,7 @@
         <v>24</v>
       </c>
       <c r="J172" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K172" t="s">
         <v>25</v>
@@ -11305,7 +11305,7 @@
         <v>25</v>
       </c>
       <c r="O172" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="P172">
         <v>82.8125</v>
@@ -11319,7 +11319,7 @@
         <v>59</v>
       </c>
       <c r="B173" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="C173" t="s">
         <v>19</v>
@@ -11331,7 +11331,7 @@
         <v>33</v>
       </c>
       <c r="F173" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="G173">
         <v>0</v>
@@ -11343,7 +11343,7 @@
         <v>24</v>
       </c>
       <c r="J173" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K173" t="s">
         <v>25</v>
@@ -11358,7 +11358,7 @@
         <v>25</v>
       </c>
       <c r="O173" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="P173">
         <v>81.66579603838262</v>
@@ -11372,7 +11372,7 @@
         <v>59</v>
       </c>
       <c r="B174" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="C174" t="s">
         <v>19</v>
@@ -11384,7 +11384,7 @@
         <v>21</v>
       </c>
       <c r="F174" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="G174">
         <v>1</v>
@@ -11396,7 +11396,7 @@
         <v>30</v>
       </c>
       <c r="J174" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K174" t="s">
         <v>25</v>
@@ -11411,7 +11411,7 @@
         <v>25</v>
       </c>
       <c r="O174" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="P174">
         <v>82.734375</v>
@@ -11425,7 +11425,7 @@
         <v>59</v>
       </c>
       <c r="B175" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="C175" t="s">
         <v>19</v>
@@ -11437,7 +11437,7 @@
         <v>33</v>
       </c>
       <c r="F175" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="G175">
         <v>1</v>
@@ -11449,7 +11449,7 @@
         <v>30</v>
       </c>
       <c r="J175" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K175" t="s">
         <v>25</v>
@@ -11464,7 +11464,7 @@
         <v>25</v>
       </c>
       <c r="O175" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="P175">
         <v>93.23432290224808</v>
@@ -11478,7 +11478,7 @@
         <v>59</v>
       </c>
       <c r="B176" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="C176" t="s">
         <v>19</v>
@@ -11490,7 +11490,7 @@
         <v>21</v>
       </c>
       <c r="F176" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="G176">
         <v>0</v>
@@ -11502,7 +11502,7 @@
         <v>24</v>
       </c>
       <c r="J176" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K176" t="s">
         <v>25</v>
@@ -11517,7 +11517,7 @@
         <v>25</v>
       </c>
       <c r="O176" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="P176">
         <v>69.57616602274948</v>
@@ -11531,7 +11531,7 @@
         <v>17</v>
       </c>
       <c r="B177" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="C177" t="s">
         <v>19</v>
@@ -11543,7 +11543,7 @@
         <v>21</v>
       </c>
       <c r="F177" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="G177">
         <v>2</v>
@@ -11555,7 +11555,7 @@
         <v>30</v>
       </c>
       <c r="J177" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K177" t="s">
         <v>25</v>
@@ -11570,7 +11570,7 @@
         <v>25</v>
       </c>
       <c r="O177" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="P177">
         <v>68.42973559023254</v>
@@ -11584,7 +11584,7 @@
         <v>17</v>
       </c>
       <c r="B178" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="C178" t="s">
         <v>19</v>
@@ -11596,7 +11596,7 @@
         <v>21</v>
       </c>
       <c r="F178" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="G178">
         <v>1</v>
@@ -11608,7 +11608,7 @@
         <v>30</v>
       </c>
       <c r="J178" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K178" t="s">
         <v>25</v>
@@ -11623,7 +11623,7 @@
         <v>25</v>
       </c>
       <c r="O178" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="P178">
         <v>71.55636404255145</v>
@@ -11637,7 +11637,7 @@
         <v>59</v>
       </c>
       <c r="B179" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="C179" t="s">
         <v>19</v>
@@ -11649,7 +11649,7 @@
         <v>21</v>
       </c>
       <c r="F179" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="G179">
         <v>1</v>
@@ -11661,7 +11661,7 @@
         <v>30</v>
       </c>
       <c r="J179" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K179" t="s">
         <v>25</v>
@@ -11676,7 +11676,7 @@
         <v>25</v>
       </c>
       <c r="O179" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="P179">
         <v>69.36772412592822</v>
@@ -11690,7 +11690,7 @@
         <v>59</v>
       </c>
       <c r="B180" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="C180" t="s">
         <v>19</v>
@@ -11702,7 +11702,7 @@
         <v>21</v>
       </c>
       <c r="F180" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="G180">
         <v>1</v>
@@ -11714,7 +11714,7 @@
         <v>30</v>
       </c>
       <c r="J180" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K180" t="s">
         <v>25</v>
@@ -11729,7 +11729,7 @@
         <v>25</v>
       </c>
       <c r="O180" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="P180">
         <v>70.93103835208767</v>
@@ -11743,7 +11743,7 @@
         <v>59</v>
       </c>
       <c r="B181" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="C181" t="s">
         <v>19</v>
@@ -11755,7 +11755,7 @@
         <v>21</v>
       </c>
       <c r="F181" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="G181">
         <v>1</v>
@@ -11767,7 +11767,7 @@
         <v>30</v>
       </c>
       <c r="J181" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K181" t="s">
         <v>25</v>
@@ -11782,7 +11782,7 @@
         <v>25</v>
       </c>
       <c r="O181" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="P181">
         <v>71.55636404255145</v>
@@ -11796,7 +11796,7 @@
         <v>59</v>
       </c>
       <c r="B182" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="C182" t="s">
         <v>19</v>
@@ -11808,7 +11808,7 @@
         <v>21</v>
       </c>
       <c r="F182" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="G182">
         <v>0</v>
@@ -11820,7 +11820,7 @@
         <v>24</v>
       </c>
       <c r="J182" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K182" t="s">
         <v>25</v>
@@ -11835,7 +11835,7 @@
         <v>25</v>
       </c>
       <c r="O182" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="P182">
         <v>70.40993361003453</v>
@@ -11849,7 +11849,7 @@
         <v>59</v>
       </c>
       <c r="B183" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="C183" t="s">
         <v>19</v>
@@ -11861,7 +11861,7 @@
         <v>21</v>
       </c>
       <c r="F183" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="G183">
         <v>0</v>
@@ -11873,7 +11873,7 @@
         <v>24</v>
       </c>
       <c r="J183" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K183" t="s">
         <v>25</v>
@@ -11888,7 +11888,7 @@
         <v>25</v>
       </c>
       <c r="O183" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="P183">
         <v>70.61837550685578</v>
@@ -11899,10 +11899,10 @@
     </row>
     <row r="184" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="B184" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="C184" t="s">
         <v>19</v>
@@ -11914,7 +11914,7 @@
         <v>21</v>
       </c>
       <c r="F184" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="G184">
         <v>0</v>
@@ -11926,7 +11926,7 @@
         <v>24</v>
       </c>
       <c r="J184" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K184" t="s">
         <v>25</v>
@@ -11941,7 +11941,7 @@
         <v>25</v>
       </c>
       <c r="O184" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="P184">
         <v>58.111861697580125</v>
@@ -11952,10 +11952,10 @@
     </row>
     <row r="185" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="B185" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="C185" t="s">
         <v>19</v>
@@ -11967,7 +11967,7 @@
         <v>21</v>
       </c>
       <c r="F185" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="G185">
         <v>1</v>
@@ -11979,7 +11979,7 @@
         <v>30</v>
       </c>
       <c r="J185" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K185" t="s">
         <v>25</v>
@@ -11994,7 +11994,7 @@
         <v>25</v>
       </c>
       <c r="O185" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="P185">
         <v>61.75959489195218</v>
@@ -12005,10 +12005,10 @@
     </row>
     <row r="186" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="B186" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="C186" t="s">
         <v>19</v>
@@ -12020,7 +12020,7 @@
         <v>21</v>
       </c>
       <c r="F186" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="G186">
         <v>1</v>
@@ -12032,7 +12032,7 @@
         <v>30</v>
       </c>
       <c r="J186" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K186" t="s">
         <v>25</v>
@@ -12047,7 +12047,7 @@
         <v>25</v>
       </c>
       <c r="O186" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="P186">
         <v>60.82160635625652</v>
@@ -12058,10 +12058,10 @@
     </row>
     <row r="187" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="B187" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="C187" t="s">
         <v>19</v>
@@ -12073,7 +12073,7 @@
         <v>21</v>
       </c>
       <c r="F187" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="G187">
         <v>1</v>
@@ -12085,7 +12085,7 @@
         <v>30</v>
       </c>
       <c r="J187" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K187" t="s">
         <v>25</v>
@@ -12100,7 +12100,7 @@
         <v>25</v>
       </c>
       <c r="O187" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="P187">
         <v>62.072257737184074</v>
@@ -12111,10 +12111,10 @@
     </row>
     <row r="188" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="B188" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="C188" t="s">
         <v>19</v>
@@ -12126,7 +12126,7 @@
         <v>21</v>
       </c>
       <c r="F188" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="G188">
         <v>0</v>
@@ -12138,7 +12138,7 @@
         <v>24</v>
       </c>
       <c r="J188" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K188" t="s">
         <v>25</v>
@@ -12153,7 +12153,7 @@
         <v>25</v>
       </c>
       <c r="O188" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="P188">
         <v>61.551152995130934</v>
@@ -12164,10 +12164,10 @@
     </row>
     <row r="189" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="B189" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="C189" t="s">
         <v>19</v>
@@ -12179,7 +12179,7 @@
         <v>21</v>
       </c>
       <c r="F189" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="G189">
         <v>1</v>
@@ -12191,7 +12191,7 @@
         <v>30</v>
       </c>
       <c r="J189" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K189" t="s">
         <v>25</v>
@@ -12206,7 +12206,7 @@
         <v>25</v>
       </c>
       <c r="O189" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="P189">
         <v>59.7793968721502</v>
@@ -12217,10 +12217,10 @@
     </row>
     <row r="190" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="B190" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="C190" t="s">
         <v>19</v>
@@ -12232,7 +12232,7 @@
         <v>21</v>
       </c>
       <c r="F190" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="G190">
         <v>0</v>
@@ -12244,7 +12244,7 @@
         <v>24</v>
       </c>
       <c r="J190" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K190" t="s">
         <v>25</v>
@@ -12259,7 +12259,7 @@
         <v>25</v>
       </c>
       <c r="O190" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="P190">
         <v>61.96803678877345</v>
@@ -12270,10 +12270,10 @@
     </row>
     <row r="191" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="B191" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="C191" t="s">
         <v>19</v>
@@ -12285,7 +12285,7 @@
         <v>21</v>
       </c>
       <c r="F191" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="G191">
         <v>1</v>
@@ -12297,7 +12297,7 @@
         <v>30</v>
       </c>
       <c r="J191" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K191" t="s">
         <v>25</v>
@@ -12312,7 +12312,7 @@
         <v>25</v>
       </c>
       <c r="O191" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="P191">
         <v>50.08684866996157</v>
@@ -12323,13 +12323,13 @@
     </row>
     <row r="192" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="B192" t="s">
         <v>25</v>
       </c>
       <c r="C192" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="D192" t="s">
         <v>25</v>
@@ -12338,7 +12338,7 @@
         <v>21</v>
       </c>
       <c r="F192" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="G192">
         <v>0</v>
@@ -12359,7 +12359,7 @@
         <v>25</v>
       </c>
       <c r="M192" t="s">
-        <v>590</v>
+        <v>226</v>
       </c>
       <c r="N192" t="s">
         <v>25</v>
@@ -12368,10 +12368,10 @@
         <v>591</v>
       </c>
       <c r="P192">
-        <v>47.15625</v>
+        <v>47.5</v>
       </c>
       <c r="Q192">
-        <v>50.10666707356771</v>
+        <v>49.20331647927297</v>
       </c>
     </row>
     <row r="193" spans="1:17" x14ac:dyDescent="0.25">
@@ -12412,7 +12412,7 @@
         <v>25</v>
       </c>
       <c r="M193" t="s">
-        <v>590</v>
+        <v>226</v>
       </c>
       <c r="N193" t="s">
         <v>25</v>

</xml_diff>